<commit_message>
release: 0.4.0 structural decoupling + sticky form UX improvements
</commit_message>
<xml_diff>
--- a/data/registry_template.xlsx
+++ b/data/registry_template.xlsx
@@ -10,10 +10,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="META" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LOOKUPS" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RULES" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1_Proyectos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C2_Aplicaciones" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C3_Componentes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C4_Runtime" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C2" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C3" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C4" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="17.34" customWidth="1" style="4" min="1" max="1"/>
@@ -651,26 +651,74 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>schema_version</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>schema_hash</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>348da3c69e16545b88f0bbeaeae28ad8a9ae28b1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>C1_label</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>C2_label</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Aplicación</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>C3_label</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Componente</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>C4_label</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Runtime</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add schema versioning, C4 reports, RBAC, dynamic labels and validation improvements
</commit_message>
<xml_diff>
--- a/data/registry_template.xlsx
+++ b/data/registry_template.xlsx
@@ -590,8 +590,10 @@
           <t>last_modified</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>46057</v>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>2026-03-16 16:08:00</t>
+        </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
@@ -658,7 +660,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>0.1.0</t>
+          <t>0.1.1</t>
         </is>
       </c>
     </row>
@@ -670,7 +672,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>348da3c69e16545b88f0bbeaeae28ad8a9ae28b1</t>
+          <t>02dcc972e13c27a5583f2c211f43b436cd8b975c</t>
         </is>
       </c>
     </row>
@@ -1882,7 +1884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9.869999999999999" customWidth="1" style="4" min="1" max="1"/>
@@ -1907,7 +1909,7 @@
     <row r="1" ht="23.85" customHeight="1" s="5">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>human_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
@@ -1993,13 +1995,18 @@
       <c r="R1" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">vulnerabilities_detected </t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>criticality</t>
         </is>
       </c>
     </row>
     <row r="2" ht="12.8" customHeight="1" s="5">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>PRJ-001</t>
+          <t>C1-001</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -2061,7 +2068,7 @@
     <row r="3" ht="12.8" customHeight="1" s="5">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>PRJ-002</t>
+          <t>C1-002</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -2160,12 +2167,12 @@
     <row r="1" ht="23.85" customHeight="1" s="5">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>c1_human_id</t>
+          <t>c1_id</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>human_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
@@ -2222,12 +2229,12 @@
     <row r="2" ht="12.8" customHeight="1" s="5">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>PRJ-001</t>
+          <t>C1-001</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>APP-001</t>
+          <t>C2-001</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -2279,12 +2286,12 @@
     <row r="3" ht="12.8" customHeight="1" s="5">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>PRJ-999</t>
+          <t>C1-999</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>APP-ORPH-1</t>
+          <t>C2-ORPH-1</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -2354,7 +2361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12.98" customWidth="1" style="4" min="1" max="1"/>
@@ -2379,12 +2386,12 @@
     <row r="1" ht="23.85" customHeight="1" s="5">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>c2_human_id</t>
+          <t>c2_id</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>human_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
@@ -2465,18 +2472,33 @@
       <c r="R1" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">vulnerabilities_detected </t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>sast_instance</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>sast_project_key</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>sast_tool</t>
         </is>
       </c>
     </row>
     <row r="2" ht="12.8" customHeight="1" s="5">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>APP-001</t>
+          <t>C2-001</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>CMP-001</t>
+          <t>C3-001</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -2538,12 +2560,12 @@
     <row r="3" ht="12.8" customHeight="1" s="5">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>APP-999</t>
+          <t>C2-999</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>CMP-ORPH-1</t>
+          <t>C3-ORPH-1</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -2613,7 +2635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12.98" customWidth="1" style="4" min="1" max="1"/>
@@ -2637,12 +2659,12 @@
     <row r="1" ht="23.85" customHeight="1" s="5">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>c3_human_id</t>
+          <t>c3_id</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>human_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
@@ -2723,18 +2745,38 @@
       <c r="R1" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">vulnerabilities_detected </t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>cspm_instance</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>cspm_resource</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>cspm_tool</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
+        <is>
+          <t>resource_group</t>
         </is>
       </c>
     </row>
     <row r="2" ht="12.8" customHeight="1" s="5">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CMP-001</t>
+          <t>C3-001</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>RUN-001</t>
+          <t>C4-001</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -2791,12 +2833,12 @@
     <row r="3" ht="12.8" customHeight="1" s="5">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CMP-999</t>
+          <t>C3-999</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>RUN-ORPH-1</t>
+          <t>C4-ORPH-1</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">

</xml_diff>